<commit_message>
Daily EOD data and reports for 2026-10-02
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261002.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261002.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.857</v>
+        <v>1.885</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.002</v>
+        <v>0.03</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.11%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>284457.12</v>
+        <v>288746.18</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>306.36</v>
+        <v>4595.43</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.51</v>
+        <v>2.55</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.01</v>
+        <v>0.03</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>1.19%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>175700</v>
+        <v>178500</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-700</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>60.74</v>
+        <v>61.21</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.48</v>
+        <v>0.95</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>1.58%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>485920</v>
+        <v>489680</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>3840</v>
+        <v>7600</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.004</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0</v>
+        <v>176.36</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-176.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>150.04</v>
+        <v>151.45</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.33</v>
+        <v>1.74</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.88</v>
+        <v>0.875</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-0.57%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>8800</v>
+        <v>8750</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>177.03</v>
+        <v>175.35</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-1.21</v>
+        <v>-2.89</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.68%</t>
+          <t>-1.62%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>708120</v>
+        <v>701400</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-4840</v>
+        <v>-11560</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.245</v>
+        <v>-0.015</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-6.12%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0</v>
+        <v>4600</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-4900</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>15.43</v>
+        <v>15.39</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.09</v>
+        <v>-0.13</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.58%</t>
+          <t>-0.84%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>46984.35</v>
+        <v>46862.55</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-274.05</v>
+        <v>-395.85</v>
       </c>
     </row>
     <row r="13">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.094</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.1</v>
+        <v>-0.006</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-6.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>564</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-600</v>
+        <v>-36</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34</v>
+        <v>34.32</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.1</v>
+        <v>0.42</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.29%</t>
+          <t>1.24%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.32</v>
+        <v>31.24</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.43</v>
+        <v>0.35</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>1.13%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>40340.16</v>
+        <v>40237.12</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>553.84</v>
+        <v>450.8</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1750321.63</v>
+        <v>1759516.21</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-9037.290000000001</v>
+        <v>157.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>